<commit_message>
New instructions w/ sample excel
</commit_message>
<xml_diff>
--- a/sample_computation_3_emp.xlsx
+++ b/sample_computation_3_emp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justi\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5FF0A5-DA28-437D-B401-D44CA52E59CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{876FC08B-5FE0-4C68-AAFC-F02A25ADEED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{E93FF709-E95F-4EF0-8785-FF148607127F}"/>
   </bookViews>
@@ -95,7 +95,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -168,14 +168,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="170" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -510,147 +513,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AE6E29E-96AD-4ECE-AC7C-115366E264FE}">
-  <dimension ref="E2:N33"/>
+  <dimension ref="A2:L27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" customWidth="1"/>
+    <col min="8" max="8" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="4.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="4.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E2" s="9" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="9"/>
-      <c r="I2" s="9" t="s">
+      <c r="F2" s="14"/>
+      <c r="H2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="9"/>
-      <c r="M2" s="9" t="s">
+      <c r="I2" s="6"/>
+      <c r="K2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="9"/>
-    </row>
-    <row r="4" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E4" s="8" t="s">
+      <c r="L2" s="6"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="I4" s="8" t="s">
+      <c r="F4" s="15"/>
+      <c r="H4" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="J4" s="8"/>
-      <c r="M4" s="8" t="s">
+      <c r="I4" s="8"/>
+      <c r="K4" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="N4" s="8"/>
-    </row>
-    <row r="5" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L4" s="8"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="9">
+        <f>SUM(F24,I24,L24)</f>
+        <v>10.125</v>
+      </c>
       <c r="E5" s="4">
         <v>1</v>
       </c>
       <c r="F5" s="7">
         <v>4</v>
       </c>
-      <c r="I5" s="4">
-        <v>1</v>
-      </c>
-      <c r="J5" s="7">
-        <v>4</v>
-      </c>
-      <c r="M5" s="4">
-        <v>1</v>
-      </c>
-      <c r="N5" s="7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" s="7">
+        <v>4</v>
+      </c>
+      <c r="K5" s="4">
+        <v>1</v>
+      </c>
+      <c r="L5" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="13">
+        <f>B5/3</f>
+        <v>3.375</v>
+      </c>
       <c r="E6" s="4">
         <v>2</v>
       </c>
       <c r="F6" s="7">
         <v>4</v>
       </c>
-      <c r="I6" s="4">
-        <v>2</v>
-      </c>
-      <c r="J6" s="7">
-        <v>2</v>
-      </c>
-      <c r="M6" s="4">
-        <v>2</v>
-      </c>
-      <c r="N6" s="7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H6" s="4">
+        <v>2</v>
+      </c>
+      <c r="I6" s="7">
+        <v>2</v>
+      </c>
+      <c r="K6" s="4">
+        <v>2</v>
+      </c>
+      <c r="L6" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="1">
+        <f>B6*0.2</f>
+        <v>0.67500000000000004</v>
+      </c>
       <c r="E7" s="4">
         <v>3</v>
       </c>
       <c r="F7" s="7">
         <v>3</v>
       </c>
-      <c r="I7" s="4">
-        <v>3</v>
-      </c>
-      <c r="J7" s="7">
-        <v>3</v>
-      </c>
-      <c r="M7" s="4">
-        <v>3</v>
-      </c>
-      <c r="N7" s="7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H7" s="4">
+        <v>3</v>
+      </c>
+      <c r="I7" s="7">
+        <v>3</v>
+      </c>
+      <c r="K7" s="4">
+        <v>3</v>
+      </c>
+      <c r="L7" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E8" s="4">
         <v>4</v>
       </c>
       <c r="F8" s="7">
         <v>3</v>
       </c>
-      <c r="I8" s="4">
-        <v>4</v>
-      </c>
-      <c r="J8" s="7">
-        <v>3</v>
-      </c>
-      <c r="M8" s="4">
-        <v>4</v>
-      </c>
-      <c r="N8" s="7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H8" s="4">
+        <v>4</v>
+      </c>
+      <c r="I8" s="7">
+        <v>3</v>
+      </c>
+      <c r="K8" s="4">
+        <v>4</v>
+      </c>
+      <c r="L8" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E9" s="4">
         <v>5</v>
       </c>
       <c r="F9" s="7">
         <v>3</v>
       </c>
-      <c r="I9" s="4">
+      <c r="H9" s="4">
         <v>5</v>
       </c>
-      <c r="J9" s="7">
-        <v>4</v>
-      </c>
-      <c r="M9" s="4">
+      <c r="I9" s="7">
+        <v>4</v>
+      </c>
+      <c r="K9" s="4">
         <v>5</v>
       </c>
-      <c r="N9" s="7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L9" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>1</v>
       </c>
@@ -658,22 +688,22 @@
         <f>SUM(F5:F9)</f>
         <v>17</v>
       </c>
-      <c r="I10" t="s">
-        <v>1</v>
-      </c>
-      <c r="J10" s="5">
-        <f>SUM(J5:J9)</f>
+      <c r="H10" t="s">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5">
+        <f>SUM(I5:I9)</f>
         <v>16</v>
       </c>
-      <c r="M10" t="s">
-        <v>1</v>
-      </c>
-      <c r="N10" s="5">
-        <f>SUM(N5:N9)</f>
+      <c r="K10" t="s">
+        <v>1</v>
+      </c>
+      <c r="L10" s="5">
+        <f>SUM(L5:L9)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="5:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>2</v>
       </c>
@@ -681,219 +711,219 @@
         <f>F10/5</f>
         <v>3.4</v>
       </c>
-      <c r="I11" t="s">
-        <v>2</v>
-      </c>
-      <c r="J11" s="3">
-        <f>J10/5</f>
+      <c r="H11" t="s">
+        <v>2</v>
+      </c>
+      <c r="I11" s="3">
+        <f>I10/5</f>
         <v>3.2</v>
       </c>
-      <c r="M11" t="s">
-        <v>2</v>
-      </c>
-      <c r="N11" s="3">
-        <f>N10/5</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="K11" t="s">
+        <v>2</v>
+      </c>
+      <c r="L11" s="3">
+        <f>L10/5</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="10">
         <f>F11*0.8</f>
         <v>2.72</v>
       </c>
-      <c r="I12" t="s">
-        <v>3</v>
-      </c>
-      <c r="J12" s="11">
-        <f>J11*0.8</f>
+      <c r="H12" t="s">
+        <v>3</v>
+      </c>
+      <c r="I12" s="10">
+        <f>I11*0.8</f>
         <v>2.5600000000000005</v>
       </c>
-      <c r="M12" t="s">
-        <v>3</v>
-      </c>
-      <c r="N12" s="12">
-        <f>N11*0.8</f>
+      <c r="K12" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="11">
+        <f>L11*0.8</f>
         <v>3.2</v>
       </c>
     </row>
-    <row r="14" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E14" s="9" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E14" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="F14" s="9"/>
-      <c r="I14" s="9" t="s">
+      <c r="F14" s="14"/>
+      <c r="H14" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="J14" s="9"/>
-      <c r="M14" s="9" t="s">
+      <c r="I14" s="6"/>
+      <c r="K14" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="N14" s="9"/>
-    </row>
-    <row r="15" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L14" s="6"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E15" s="4">
         <v>1</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
-      <c r="I15" s="4">
-        <v>1</v>
-      </c>
-      <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="M15" s="4">
-        <v>1</v>
-      </c>
-      <c r="N15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H15" s="4">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="K15" s="4">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E16" s="4">
         <v>2</v>
       </c>
       <c r="F16">
         <v>4</v>
       </c>
-      <c r="I16" s="4">
-        <v>2</v>
-      </c>
-      <c r="J16">
-        <v>1</v>
-      </c>
-      <c r="M16" s="4">
-        <v>2</v>
-      </c>
-      <c r="N16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H16" s="4">
+        <v>2</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="K16" s="4">
+        <v>2</v>
+      </c>
+      <c r="L16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E17" s="4">
         <v>3</v>
       </c>
       <c r="F17">
         <v>2</v>
       </c>
-      <c r="I17" s="4">
-        <v>3</v>
-      </c>
-      <c r="J17">
-        <v>4</v>
-      </c>
-      <c r="M17" s="4">
-        <v>3</v>
-      </c>
-      <c r="N17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H17" s="4">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>4</v>
+      </c>
+      <c r="K17" s="4">
+        <v>3</v>
+      </c>
+      <c r="L17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E18" s="4">
         <v>4</v>
       </c>
       <c r="F18">
         <v>4</v>
       </c>
-      <c r="I18" s="4">
-        <v>4</v>
-      </c>
-      <c r="J18">
-        <v>4</v>
-      </c>
-      <c r="M18" s="4">
-        <v>4</v>
-      </c>
-      <c r="N18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="H18" s="4">
+        <v>4</v>
+      </c>
+      <c r="I18">
+        <v>4</v>
+      </c>
+      <c r="K18" s="4">
+        <v>4</v>
+      </c>
+      <c r="L18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E19" s="4">
         <v>5</v>
       </c>
       <c r="F19">
         <v>4</v>
       </c>
-      <c r="I19" s="4">
+      <c r="H19" s="4">
         <v>5</v>
       </c>
-      <c r="J19">
-        <v>4</v>
-      </c>
-      <c r="M19" s="4">
+      <c r="I19">
+        <v>4</v>
+      </c>
+      <c r="K19" s="4">
         <v>5</v>
       </c>
-      <c r="N19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E20" s="4">
         <v>6</v>
       </c>
       <c r="F20">
         <v>3</v>
       </c>
-      <c r="I20" s="4">
+      <c r="H20" s="4">
         <v>6</v>
       </c>
-      <c r="J20">
-        <v>4</v>
-      </c>
-      <c r="M20" s="4">
+      <c r="I20">
+        <v>4</v>
+      </c>
+      <c r="K20" s="4">
         <v>6</v>
       </c>
-      <c r="N20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E21" s="4">
         <v>7</v>
       </c>
       <c r="F21">
         <v>2</v>
       </c>
-      <c r="I21" s="4">
+      <c r="H21" s="4">
         <v>7</v>
       </c>
-      <c r="J21">
-        <v>4</v>
-      </c>
-      <c r="M21" s="4">
+      <c r="I21">
+        <v>4</v>
+      </c>
+      <c r="K21" s="4">
         <v>7</v>
       </c>
-      <c r="N21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E22" s="4">
         <v>8</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
-      <c r="I22" s="4">
+      <c r="H22" s="4">
         <v>8</v>
       </c>
-      <c r="J22">
-        <v>4</v>
-      </c>
-      <c r="M22" s="4">
+      <c r="I22">
+        <v>4</v>
+      </c>
+      <c r="K22" s="4">
         <v>8</v>
       </c>
-      <c r="N22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
         <v>4</v>
       </c>
@@ -901,68 +931,68 @@
         <f>SUM(F15:F22)</f>
         <v>23</v>
       </c>
-      <c r="I23" t="s">
-        <v>4</v>
-      </c>
-      <c r="J23" s="5">
-        <f>SUM(J15:J22)</f>
+      <c r="H23" t="s">
+        <v>4</v>
+      </c>
+      <c r="I23" s="5">
+        <f>SUM(I15:I22)</f>
         <v>26</v>
       </c>
-      <c r="M23" t="s">
-        <v>4</v>
-      </c>
-      <c r="N23" s="5">
-        <f>SUM(N15:N22)</f>
+      <c r="K23" t="s">
+        <v>4</v>
+      </c>
+      <c r="L23" s="5">
+        <f>SUM(L15:L22)</f>
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="5:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="9">
         <f>F23/8</f>
         <v>2.875</v>
       </c>
-      <c r="I24" t="s">
+      <c r="H24" t="s">
         <v>6</v>
       </c>
-      <c r="J24" s="3">
-        <f>J23/8</f>
+      <c r="I24" s="3">
+        <f>I23/8</f>
         <v>3.25</v>
       </c>
-      <c r="M24" t="s">
+      <c r="K24" t="s">
         <v>6</v>
       </c>
-      <c r="N24" s="13">
-        <f>N23/8</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="L24" s="12">
+        <f>L23/8</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
         <v>7</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="10">
         <f>F24*0.2</f>
         <v>0.57500000000000007</v>
       </c>
-      <c r="I25" t="s">
+      <c r="H25" t="s">
         <v>7</v>
       </c>
-      <c r="J25" s="11">
-        <f>J24*0.2</f>
+      <c r="I25" s="10">
+        <f>I24*0.2</f>
         <v>0.65</v>
       </c>
-      <c r="M25" t="s">
+      <c r="K25" t="s">
         <v>7</v>
       </c>
-      <c r="N25" s="12">
-        <f>N24*0.2</f>
+      <c r="L25" s="11">
+        <f>L24*0.2</f>
         <v>0.8</v>
       </c>
     </row>
-    <row r="27" spans="5:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E27" t="s">
         <v>8</v>
       </c>
@@ -970,64 +1000,26 @@
         <f>SUM(F12,F25)</f>
         <v>3.2950000000000004</v>
       </c>
-      <c r="I27" t="s">
+      <c r="H27" t="s">
         <v>8</v>
       </c>
-      <c r="J27" s="2">
-        <f>SUM(J12,J25)</f>
+      <c r="I27" s="2">
+        <f>SUM(I12,I25)</f>
         <v>3.2100000000000004</v>
       </c>
-      <c r="M27" t="s">
+      <c r="K27" t="s">
         <v>8</v>
       </c>
-      <c r="N27" s="2">
-        <f>SUM(N12,N25)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="I30" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="H31" t="s">
-        <v>13</v>
-      </c>
-      <c r="I31" s="10">
-        <f>SUM(F24,J24,N24)</f>
-        <v>10.125</v>
-      </c>
-    </row>
-    <row r="32" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="H32" t="s">
-        <v>14</v>
-      </c>
-      <c r="I32" s="14">
-        <f>I31/3</f>
-        <v>3.375</v>
-      </c>
-    </row>
-    <row r="33" spans="8:9" x14ac:dyDescent="0.25">
-      <c r="H33" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" s="1">
-        <f>I32*0.2</f>
-        <v>0.67500000000000004</v>
+      <c r="L27" s="2">
+        <f>SUM(L12,L25)</f>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="M14:N14"/>
+  <mergeCells count="3">
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I14:J14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>